<commit_message>
Regenerate ER model — exclude Coming soon menus
- Drop entities mapped to 'Coming soon' menus from all sheets: payment,
  debt, report, evaluation, document, notification, knowledge_article
  (and their orphaned enums payment_status, notification_channel)
- 29 entities remain (28 base + module_progress view)
- Refresh module_template / module CRUD points for the new
  create-in-templates / instantiate-in-modules flow

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01C1rM739bFjpxKpAnsLyCHD
</commit_message>
<xml_diff>
--- a/SJA_ER_Model.xlsx
+++ b/SJA_ER_Model.xlsx
@@ -15,11 +15,11 @@
     <sheet name="Enums" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Entities'!$A$1:$F$37</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Attributes'!$A$1:$G$312</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Relationships'!$A$1:$G$67</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'CRUD Matrix'!$A$1:$F$37</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Enums'!$A$1:$C$15</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Entities'!$A$1:$F$30</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Attributes'!$A$1:$G$263</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Relationships'!$A$1:$G$60</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'CRUD Matrix'!$A$1:$F$30</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Enums'!$A$1:$C$13</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -658,7 +658,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -699,79 +699,91 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>36 (31 base tables + 3 planned + 2 derived views)</t>
+          <t>29 (28 base tables + 1 derived view)</t>
         </is>
       </c>
     </row>
     <row r="6" ht="15" customHeight="1">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>Key convention</t>
+          <t>Scope</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Every entity has a surrogate id bigint PRIMARY KEY (GENERATED ALWAYS AS IDENTITY). Views have no id.</t>
+          <t>Excludes modules mapped to 'Coming soon' menus: Payments, Debts, Reports, Evaluations, Documents, Notifications, AI/Knowledge Base.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="15" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>Foreign keys</t>
+          <t>Key convention</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>bigint columns ending _id referencing &lt;table&gt;(id).</t>
+          <t>Every entity has a surrogate id bigint PRIMARY KEY (GENERATED ALWAYS AS IDENTITY). Views have no id.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="15" customHeight="1">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>Enums</t>
+          <t>Foreign keys</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Modeled as PostgreSQL ENUM types — see the 'Enums' sheet.</t>
+          <t>bigint columns ending _id referencing &lt;table&gt;(id).</t>
         </is>
       </c>
     </row>
     <row r="9" ht="15" customHeight="1">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>Derived note</t>
+          <t>Enums</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>trainer total/monthly hours = SUM(lesson duration) — computed, not stored.</t>
+          <t>Modeled as PostgreSQL ENUM types — see the 'Enums' sheet.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="15" customHeight="1">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>Sheets</t>
+          <t>Derived note</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>Overview · Entities · Attributes · Relationships · CRUD Matrix · Enums</t>
+          <t>trainer total/monthly hours = SUM(lesson duration) — computed, not stored.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="15" customHeight="1">
       <c r="A11" s="3" t="inlineStr">
         <is>
+          <t>Sheets</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>Overview · Entities · Attributes · Relationships · CRUD Matrix · Enums</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="15" customHeight="1">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
           <t>CRUD legend</t>
         </is>
       </c>
-      <c r="B11" s="4" t="inlineStr">
-        <is>
-          <t>C=Create R=Read U=Update D=Delete. 'NONE' = no CRUD point in the current system (planned or derived).</t>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>C=Create R=Read U=Update D=Delete. 'NONE' = no CRUD point in the current system (e.g. reference or derived).</t>
         </is>
       </c>
     </row>
@@ -786,7 +798,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F37"/>
+  <dimension ref="A1:F30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1645,7 +1657,7 @@
       </c>
       <c r="B29" s="11" t="inlineStr">
         <is>
-          <t>payment</t>
+          <t>subscription</t>
         </is>
       </c>
       <c r="C29" s="12" t="inlineStr">
@@ -1665,7 +1677,7 @@
       </c>
       <c r="F29" s="12" t="inlineStr">
         <is>
-          <t>Tuition payment (Fina integration).</t>
+          <t>Recurring subscription the parent activates.</t>
         </is>
       </c>
     </row>
@@ -1675,242 +1687,32 @@
       </c>
       <c r="B30" s="7" t="inlineStr">
         <is>
-          <t>subscription</t>
+          <t>module_progress</t>
         </is>
       </c>
       <c r="C30" s="8" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>Derived</t>
         </is>
       </c>
       <c r="D30" s="9" t="inlineStr">
         <is>
-          <t>id</t>
-        </is>
-      </c>
-      <c r="E30" s="6" t="inlineStr">
-        <is>
-          <t>Yes</t>
+          <t>(composite — VIEW)</t>
+        </is>
+      </c>
+      <c r="E30" s="14" t="inlineStr">
+        <is>
+          <t>No</t>
         </is>
       </c>
       <c r="F30" s="8" t="inlineStr">
         <is>
-          <t>Recurring subscription the parent activates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="10" t="n">
-        <v>30</v>
-      </c>
-      <c r="B31" s="11" t="inlineStr">
-        <is>
-          <t>document</t>
-        </is>
-      </c>
-      <c r="C31" s="12" t="inlineStr">
-        <is>
-          <t>Documents</t>
-        </is>
-      </c>
-      <c r="D31" s="13" t="inlineStr">
-        <is>
-          <t>id</t>
-        </is>
-      </c>
-      <c r="E31" s="10" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="F31" s="12" t="inlineStr">
-        <is>
-          <t>Uploaded document (contract, certificate, …).</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="6" t="n">
-        <v>31</v>
-      </c>
-      <c r="B32" s="7" t="inlineStr">
-        <is>
-          <t>notification</t>
-        </is>
-      </c>
-      <c r="C32" s="8" t="inlineStr">
-        <is>
-          <t>Communication</t>
-        </is>
-      </c>
-      <c r="D32" s="9" t="inlineStr">
-        <is>
-          <t>id</t>
-        </is>
-      </c>
-      <c r="E32" s="6" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="F32" s="8" t="inlineStr">
-        <is>
-          <t>System notification / reminder to a user.</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="10" t="n">
-        <v>32</v>
-      </c>
-      <c r="B33" s="11" t="inlineStr">
-        <is>
-          <t>report</t>
-        </is>
-      </c>
-      <c r="C33" s="12" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="D33" s="13" t="inlineStr">
-        <is>
-          <t>id</t>
-        </is>
-      </c>
-      <c r="E33" s="14" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F33" s="12" t="inlineStr">
-        <is>
-          <t>Reporting output (templates, schedule, archive).</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="6" t="n">
-        <v>33</v>
-      </c>
-      <c r="B34" s="7" t="inlineStr">
-        <is>
-          <t>evaluation</t>
-        </is>
-      </c>
-      <c r="C34" s="8" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="D34" s="9" t="inlineStr">
-        <is>
-          <t>id</t>
-        </is>
-      </c>
-      <c r="E34" s="14" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F34" s="8" t="inlineStr">
-        <is>
-          <t>Evaluations of trainers/students/groups.</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="10" t="n">
-        <v>34</v>
-      </c>
-      <c r="B35" s="11" t="inlineStr">
-        <is>
-          <t>knowledge_article</t>
-        </is>
-      </c>
-      <c r="C35" s="12" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="D35" s="13" t="inlineStr">
-        <is>
-          <t>id</t>
-        </is>
-      </c>
-      <c r="E35" s="14" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F35" s="12" t="inlineStr">
-        <is>
-          <t>AI / Knowledge Base article.</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="6" t="n">
-        <v>35</v>
-      </c>
-      <c r="B36" s="7" t="inlineStr">
-        <is>
-          <t>module_progress</t>
-        </is>
-      </c>
-      <c r="C36" s="8" t="inlineStr">
-        <is>
-          <t>Derived</t>
-        </is>
-      </c>
-      <c r="D36" s="9" t="inlineStr">
-        <is>
-          <t>(composite — VIEW)</t>
-        </is>
-      </c>
-      <c r="E36" s="14" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F36" s="8" t="inlineStr">
-        <is>
           <t>VIEW: student progress per module (computed).</t>
         </is>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="10" t="n">
-        <v>36</v>
-      </c>
-      <c r="B37" s="11" t="inlineStr">
-        <is>
-          <t>debt</t>
-        </is>
-      </c>
-      <c r="C37" s="12" t="inlineStr">
-        <is>
-          <t>Derived</t>
-        </is>
-      </c>
-      <c r="D37" s="13" t="inlineStr">
-        <is>
-          <t>(composite — VIEW)</t>
-        </is>
-      </c>
-      <c r="E37" s="14" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F37" s="12" t="inlineStr">
-        <is>
-          <t>VIEW: outstanding balance per student (computed from payments).</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:F37"/>
+  <autoFilter ref="A1:F30"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1921,7 +1723,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G312"/>
+  <dimension ref="A1:G263"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -7793,7 +7595,7 @@
     <row r="250">
       <c r="A250" s="15" t="inlineStr">
         <is>
-          <t>payment</t>
+          <t>subscription</t>
         </is>
       </c>
       <c r="B250" s="16" t="inlineStr">
@@ -7852,7 +7654,7 @@
       <c r="A252" s="3" t="inlineStr"/>
       <c r="B252" s="17" t="inlineStr">
         <is>
-          <t>semester_id</t>
+          <t>parent_id</t>
         </is>
       </c>
       <c r="C252" s="17" t="inlineStr">
@@ -7867,7 +7669,7 @@
       </c>
       <c r="E252" s="19" t="inlineStr">
         <is>
-          <t>semester(id)</t>
+          <t>parent(id)</t>
         </is>
       </c>
       <c r="F252" s="23" t="inlineStr">
@@ -7881,12 +7683,12 @@
       <c r="A253" s="3" t="inlineStr"/>
       <c r="B253" s="17" t="inlineStr">
         <is>
-          <t>amount</t>
-        </is>
-      </c>
-      <c r="C253" s="21" t="inlineStr">
-        <is>
-          <t>numeric(10,2)</t>
+          <t>is_active</t>
+        </is>
+      </c>
+      <c r="C253" s="17" t="inlineStr">
+        <is>
+          <t>boolean</t>
         </is>
       </c>
       <c r="D253" s="22" t="inlineStr"/>
@@ -7902,116 +7704,108 @@
       <c r="A254" s="3" t="inlineStr"/>
       <c r="B254" s="17" t="inlineStr">
         <is>
-          <t>currency</t>
+          <t>activated_at</t>
         </is>
       </c>
       <c r="C254" s="21" t="inlineStr">
         <is>
-          <t>char(3)</t>
+          <t>timestamptz</t>
         </is>
       </c>
       <c r="D254" s="22" t="inlineStr"/>
       <c r="E254" s="19" t="inlineStr"/>
-      <c r="F254" s="20" t="inlineStr">
-        <is>
-          <t>NOT NULL</t>
-        </is>
-      </c>
-      <c r="G254" s="4" t="inlineStr">
-        <is>
-          <t>Default 'GEL'</t>
-        </is>
-      </c>
+      <c r="F254" s="23" t="inlineStr">
+        <is>
+          <t>NULL</t>
+        </is>
+      </c>
+      <c r="G254" s="4" t="inlineStr"/>
     </row>
     <row r="255">
       <c r="A255" s="3" t="inlineStr"/>
       <c r="B255" s="17" t="inlineStr">
         <is>
-          <t>status</t>
+          <t>amount</t>
         </is>
       </c>
       <c r="C255" s="21" t="inlineStr">
         <is>
-          <t>payment_status</t>
+          <t>numeric(10,2)</t>
         </is>
       </c>
       <c r="D255" s="22" t="inlineStr"/>
       <c r="E255" s="19" t="inlineStr"/>
-      <c r="F255" s="20" t="inlineStr">
-        <is>
-          <t>NOT NULL</t>
-        </is>
-      </c>
-      <c r="G255" s="4" t="inlineStr">
-        <is>
-          <t>ENUM: paid/pending/unallocated/overdue</t>
-        </is>
-      </c>
+      <c r="F255" s="23" t="inlineStr">
+        <is>
+          <t>NULL</t>
+        </is>
+      </c>
+      <c r="G255" s="4" t="inlineStr"/>
     </row>
     <row r="256">
       <c r="A256" s="3" t="inlineStr"/>
       <c r="B256" s="17" t="inlineStr">
         <is>
-          <t>due_date</t>
-        </is>
-      </c>
-      <c r="C256" s="17" t="inlineStr">
-        <is>
-          <t>date</t>
+          <t>created_at</t>
+        </is>
+      </c>
+      <c r="C256" s="21" t="inlineStr">
+        <is>
+          <t>timestamptz</t>
         </is>
       </c>
       <c r="D256" s="22" t="inlineStr"/>
       <c r="E256" s="19" t="inlineStr"/>
-      <c r="F256" s="23" t="inlineStr">
-        <is>
-          <t>NULL</t>
+      <c r="F256" s="20" t="inlineStr">
+        <is>
+          <t>NOT NULL</t>
         </is>
       </c>
       <c r="G256" s="4" t="inlineStr"/>
     </row>
-    <row r="257">
-      <c r="A257" s="3" t="inlineStr"/>
-      <c r="B257" s="17" t="inlineStr">
-        <is>
-          <t>paid_at</t>
-        </is>
-      </c>
-      <c r="C257" s="21" t="inlineStr">
-        <is>
-          <t>timestamptz</t>
-        </is>
-      </c>
-      <c r="D257" s="22" t="inlineStr"/>
-      <c r="E257" s="19" t="inlineStr"/>
-      <c r="F257" s="23" t="inlineStr">
-        <is>
-          <t>NULL</t>
-        </is>
-      </c>
-      <c r="G257" s="4" t="inlineStr"/>
+    <row r="257" ht="4" customHeight="1">
+      <c r="A257" s="25" t="n"/>
+      <c r="B257" s="25" t="n"/>
+      <c r="C257" s="25" t="n"/>
+      <c r="D257" s="25" t="n"/>
+      <c r="E257" s="25" t="n"/>
+      <c r="F257" s="25" t="n"/>
+      <c r="G257" s="25" t="n"/>
     </row>
     <row r="258">
-      <c r="A258" s="3" t="inlineStr"/>
+      <c r="A258" s="15" t="inlineStr">
+        <is>
+          <t>module_progress</t>
+        </is>
+      </c>
       <c r="B258" s="17" t="inlineStr">
         <is>
-          <t>external_ref</t>
-        </is>
-      </c>
-      <c r="C258" s="21" t="inlineStr">
-        <is>
-          <t>varchar(80)</t>
-        </is>
-      </c>
-      <c r="D258" s="22" t="inlineStr"/>
-      <c r="E258" s="19" t="inlineStr"/>
-      <c r="F258" s="23" t="inlineStr">
-        <is>
-          <t>NULL</t>
+          <t>student_id</t>
+        </is>
+      </c>
+      <c r="C258" s="17" t="inlineStr">
+        <is>
+          <t>bigint</t>
+        </is>
+      </c>
+      <c r="D258" s="24" t="inlineStr">
+        <is>
+          <t>FK</t>
+        </is>
+      </c>
+      <c r="E258" s="19" t="inlineStr">
+        <is>
+          <t>student(id)</t>
+        </is>
+      </c>
+      <c r="F258" s="20" t="inlineStr">
+        <is>
+          <t>NOT NULL</t>
         </is>
       </c>
       <c r="G258" s="4" t="inlineStr">
         <is>
-          <t>Fina reference</t>
+          <t>Part of composite key</t>
         </is>
       </c>
     </row>
@@ -8019,1206 +7813,121 @@
       <c r="A259" s="3" t="inlineStr"/>
       <c r="B259" s="17" t="inlineStr">
         <is>
-          <t>created_at</t>
-        </is>
-      </c>
-      <c r="C259" s="21" t="inlineStr">
-        <is>
-          <t>timestamptz</t>
-        </is>
-      </c>
-      <c r="D259" s="22" t="inlineStr"/>
-      <c r="E259" s="19" t="inlineStr"/>
+          <t>module_id</t>
+        </is>
+      </c>
+      <c r="C259" s="17" t="inlineStr">
+        <is>
+          <t>bigint</t>
+        </is>
+      </c>
+      <c r="D259" s="24" t="inlineStr">
+        <is>
+          <t>FK</t>
+        </is>
+      </c>
+      <c r="E259" s="19" t="inlineStr">
+        <is>
+          <t>module(id)</t>
+        </is>
+      </c>
       <c r="F259" s="20" t="inlineStr">
         <is>
           <t>NOT NULL</t>
         </is>
       </c>
-      <c r="G259" s="4" t="inlineStr"/>
-    </row>
-    <row r="260" ht="4" customHeight="1">
-      <c r="A260" s="25" t="n"/>
-      <c r="B260" s="25" t="n"/>
-      <c r="C260" s="25" t="n"/>
-      <c r="D260" s="25" t="n"/>
-      <c r="E260" s="25" t="n"/>
-      <c r="F260" s="25" t="n"/>
-      <c r="G260" s="25" t="n"/>
+      <c r="G259" s="4" t="inlineStr">
+        <is>
+          <t>Part of composite key</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" s="3" t="inlineStr"/>
+      <c r="B260" s="17" t="inlineStr">
+        <is>
+          <t>completed_lectures</t>
+        </is>
+      </c>
+      <c r="C260" s="17" t="inlineStr">
+        <is>
+          <t>integer</t>
+        </is>
+      </c>
+      <c r="D260" s="22" t="inlineStr"/>
+      <c r="E260" s="19" t="inlineStr"/>
+      <c r="F260" s="20" t="inlineStr">
+        <is>
+          <t>NOT NULL</t>
+        </is>
+      </c>
+      <c r="G260" s="4" t="inlineStr">
+        <is>
+          <t>Computed</t>
+        </is>
+      </c>
     </row>
     <row r="261">
-      <c r="A261" s="15" t="inlineStr">
-        <is>
-          <t>subscription</t>
-        </is>
-      </c>
-      <c r="B261" s="16" t="inlineStr">
-        <is>
-          <t>id</t>
+      <c r="A261" s="3" t="inlineStr"/>
+      <c r="B261" s="17" t="inlineStr">
+        <is>
+          <t>total_lectures</t>
         </is>
       </c>
       <c r="C261" s="17" t="inlineStr">
         <is>
-          <t>bigint</t>
-        </is>
-      </c>
-      <c r="D261" s="18" t="inlineStr">
-        <is>
-          <t>PK</t>
-        </is>
-      </c>
+          <t>integer</t>
+        </is>
+      </c>
+      <c r="D261" s="22" t="inlineStr"/>
       <c r="E261" s="19" t="inlineStr"/>
       <c r="F261" s="20" t="inlineStr">
         <is>
           <t>NOT NULL</t>
         </is>
       </c>
-      <c r="G261" s="4" t="inlineStr"/>
+      <c r="G261" s="4" t="inlineStr">
+        <is>
+          <t>Computed</t>
+        </is>
+      </c>
     </row>
     <row r="262">
       <c r="A262" s="3" t="inlineStr"/>
       <c r="B262" s="17" t="inlineStr">
         <is>
-          <t>student_id</t>
-        </is>
-      </c>
-      <c r="C262" s="17" t="inlineStr">
-        <is>
-          <t>bigint</t>
-        </is>
-      </c>
-      <c r="D262" s="24" t="inlineStr">
-        <is>
-          <t>FK</t>
-        </is>
-      </c>
-      <c r="E262" s="19" t="inlineStr">
-        <is>
-          <t>student(id)</t>
-        </is>
-      </c>
+          <t>progress_pct</t>
+        </is>
+      </c>
+      <c r="C262" s="21" t="inlineStr">
+        <is>
+          <t>numeric(5,2)</t>
+        </is>
+      </c>
+      <c r="D262" s="22" t="inlineStr"/>
+      <c r="E262" s="19" t="inlineStr"/>
       <c r="F262" s="20" t="inlineStr">
         <is>
           <t>NOT NULL</t>
         </is>
       </c>
-      <c r="G262" s="4" t="inlineStr"/>
-    </row>
-    <row r="263">
-      <c r="A263" s="3" t="inlineStr"/>
-      <c r="B263" s="17" t="inlineStr">
-        <is>
-          <t>parent_id</t>
-        </is>
-      </c>
-      <c r="C263" s="17" t="inlineStr">
-        <is>
-          <t>bigint</t>
-        </is>
-      </c>
-      <c r="D263" s="24" t="inlineStr">
-        <is>
-          <t>FK</t>
-        </is>
-      </c>
-      <c r="E263" s="19" t="inlineStr">
-        <is>
-          <t>parent(id)</t>
-        </is>
-      </c>
-      <c r="F263" s="23" t="inlineStr">
-        <is>
-          <t>NULL</t>
-        </is>
-      </c>
-      <c r="G263" s="4" t="inlineStr"/>
-    </row>
-    <row r="264">
-      <c r="A264" s="3" t="inlineStr"/>
-      <c r="B264" s="17" t="inlineStr">
-        <is>
-          <t>is_active</t>
-        </is>
-      </c>
-      <c r="C264" s="17" t="inlineStr">
-        <is>
-          <t>boolean</t>
-        </is>
-      </c>
-      <c r="D264" s="22" t="inlineStr"/>
-      <c r="E264" s="19" t="inlineStr"/>
-      <c r="F264" s="20" t="inlineStr">
-        <is>
-          <t>NOT NULL</t>
-        </is>
-      </c>
-      <c r="G264" s="4" t="inlineStr"/>
-    </row>
-    <row r="265">
-      <c r="A265" s="3" t="inlineStr"/>
-      <c r="B265" s="17" t="inlineStr">
-        <is>
-          <t>activated_at</t>
-        </is>
-      </c>
-      <c r="C265" s="21" t="inlineStr">
-        <is>
-          <t>timestamptz</t>
-        </is>
-      </c>
-      <c r="D265" s="22" t="inlineStr"/>
-      <c r="E265" s="19" t="inlineStr"/>
-      <c r="F265" s="23" t="inlineStr">
-        <is>
-          <t>NULL</t>
-        </is>
-      </c>
-      <c r="G265" s="4" t="inlineStr"/>
-    </row>
-    <row r="266">
-      <c r="A266" s="3" t="inlineStr"/>
-      <c r="B266" s="17" t="inlineStr">
-        <is>
-          <t>amount</t>
-        </is>
-      </c>
-      <c r="C266" s="21" t="inlineStr">
-        <is>
-          <t>numeric(10,2)</t>
-        </is>
-      </c>
-      <c r="D266" s="22" t="inlineStr"/>
-      <c r="E266" s="19" t="inlineStr"/>
-      <c r="F266" s="23" t="inlineStr">
-        <is>
-          <t>NULL</t>
-        </is>
-      </c>
-      <c r="G266" s="4" t="inlineStr"/>
-    </row>
-    <row r="267">
-      <c r="A267" s="3" t="inlineStr"/>
-      <c r="B267" s="17" t="inlineStr">
-        <is>
-          <t>created_at</t>
-        </is>
-      </c>
-      <c r="C267" s="21" t="inlineStr">
-        <is>
-          <t>timestamptz</t>
-        </is>
-      </c>
-      <c r="D267" s="22" t="inlineStr"/>
-      <c r="E267" s="19" t="inlineStr"/>
-      <c r="F267" s="20" t="inlineStr">
-        <is>
-          <t>NOT NULL</t>
-        </is>
-      </c>
-      <c r="G267" s="4" t="inlineStr"/>
-    </row>
-    <row r="268" ht="4" customHeight="1">
-      <c r="A268" s="25" t="n"/>
-      <c r="B268" s="25" t="n"/>
-      <c r="C268" s="25" t="n"/>
-      <c r="D268" s="25" t="n"/>
-      <c r="E268" s="25" t="n"/>
-      <c r="F268" s="25" t="n"/>
-      <c r="G268" s="25" t="n"/>
-    </row>
-    <row r="269">
-      <c r="A269" s="15" t="inlineStr">
-        <is>
-          <t>document</t>
-        </is>
-      </c>
-      <c r="B269" s="16" t="inlineStr">
-        <is>
-          <t>id</t>
-        </is>
-      </c>
-      <c r="C269" s="17" t="inlineStr">
-        <is>
-          <t>bigint</t>
-        </is>
-      </c>
-      <c r="D269" s="18" t="inlineStr">
-        <is>
-          <t>PK</t>
-        </is>
-      </c>
-      <c r="E269" s="19" t="inlineStr"/>
-      <c r="F269" s="20" t="inlineStr">
-        <is>
-          <t>NOT NULL</t>
-        </is>
-      </c>
-      <c r="G269" s="4" t="inlineStr"/>
-    </row>
-    <row r="270">
-      <c r="A270" s="3" t="inlineStr"/>
-      <c r="B270" s="17" t="inlineStr">
-        <is>
-          <t>owner_user_id</t>
-        </is>
-      </c>
-      <c r="C270" s="17" t="inlineStr">
-        <is>
-          <t>bigint</t>
-        </is>
-      </c>
-      <c r="D270" s="24" t="inlineStr">
-        <is>
-          <t>FK</t>
-        </is>
-      </c>
-      <c r="E270" s="19" t="inlineStr">
-        <is>
-          <t>app_user(id)</t>
-        </is>
-      </c>
-      <c r="F270" s="23" t="inlineStr">
-        <is>
-          <t>NULL</t>
-        </is>
-      </c>
-      <c r="G270" s="4" t="inlineStr"/>
-    </row>
-    <row r="271">
-      <c r="A271" s="3" t="inlineStr"/>
-      <c r="B271" s="17" t="inlineStr">
-        <is>
-          <t>student_id</t>
-        </is>
-      </c>
-      <c r="C271" s="17" t="inlineStr">
-        <is>
-          <t>bigint</t>
-        </is>
-      </c>
-      <c r="D271" s="24" t="inlineStr">
-        <is>
-          <t>FK</t>
-        </is>
-      </c>
-      <c r="E271" s="19" t="inlineStr">
-        <is>
-          <t>student(id)</t>
-        </is>
-      </c>
-      <c r="F271" s="23" t="inlineStr">
-        <is>
-          <t>NULL</t>
-        </is>
-      </c>
-      <c r="G271" s="4" t="inlineStr"/>
-    </row>
-    <row r="272">
-      <c r="A272" s="3" t="inlineStr"/>
-      <c r="B272" s="17" t="inlineStr">
-        <is>
-          <t>doc_type</t>
-        </is>
-      </c>
-      <c r="C272" s="21" t="inlineStr">
-        <is>
-          <t>varchar(60)</t>
-        </is>
-      </c>
-      <c r="D272" s="22" t="inlineStr"/>
-      <c r="E272" s="19" t="inlineStr"/>
-      <c r="F272" s="20" t="inlineStr">
-        <is>
-          <t>NOT NULL</t>
-        </is>
-      </c>
-      <c r="G272" s="4" t="inlineStr">
-        <is>
-          <t>contract/document/certificate/other</t>
-        </is>
-      </c>
-    </row>
-    <row r="273">
-      <c r="A273" s="3" t="inlineStr"/>
-      <c r="B273" s="17" t="inlineStr">
-        <is>
-          <t>title</t>
-        </is>
-      </c>
-      <c r="C273" s="21" t="inlineStr">
-        <is>
-          <t>varchar(160)</t>
-        </is>
-      </c>
-      <c r="D273" s="22" t="inlineStr"/>
-      <c r="E273" s="19" t="inlineStr"/>
-      <c r="F273" s="23" t="inlineStr">
-        <is>
-          <t>NULL</t>
-        </is>
-      </c>
-      <c r="G273" s="4" t="inlineStr"/>
-    </row>
-    <row r="274">
-      <c r="A274" s="3" t="inlineStr"/>
-      <c r="B274" s="17" t="inlineStr">
-        <is>
-          <t>file_url</t>
-        </is>
-      </c>
-      <c r="C274" s="21" t="inlineStr">
-        <is>
-          <t>varchar(500)</t>
-        </is>
-      </c>
-      <c r="D274" s="22" t="inlineStr"/>
-      <c r="E274" s="19" t="inlineStr"/>
-      <c r="F274" s="20" t="inlineStr">
-        <is>
-          <t>NOT NULL</t>
-        </is>
-      </c>
-      <c r="G274" s="4" t="inlineStr"/>
-    </row>
-    <row r="275">
-      <c r="A275" s="3" t="inlineStr"/>
-      <c r="B275" s="17" t="inlineStr">
-        <is>
-          <t>uploaded_by</t>
-        </is>
-      </c>
-      <c r="C275" s="17" t="inlineStr">
-        <is>
-          <t>bigint</t>
-        </is>
-      </c>
-      <c r="D275" s="24" t="inlineStr">
-        <is>
-          <t>FK</t>
-        </is>
-      </c>
-      <c r="E275" s="19" t="inlineStr">
-        <is>
-          <t>app_user(id)</t>
-        </is>
-      </c>
-      <c r="F275" s="23" t="inlineStr">
-        <is>
-          <t>NULL</t>
-        </is>
-      </c>
-      <c r="G275" s="4" t="inlineStr"/>
-    </row>
-    <row r="276">
-      <c r="A276" s="3" t="inlineStr"/>
-      <c r="B276" s="17" t="inlineStr">
-        <is>
-          <t>created_at</t>
-        </is>
-      </c>
-      <c r="C276" s="21" t="inlineStr">
-        <is>
-          <t>timestamptz</t>
-        </is>
-      </c>
-      <c r="D276" s="22" t="inlineStr"/>
-      <c r="E276" s="19" t="inlineStr"/>
-      <c r="F276" s="20" t="inlineStr">
-        <is>
-          <t>NOT NULL</t>
-        </is>
-      </c>
-      <c r="G276" s="4" t="inlineStr"/>
-    </row>
-    <row r="277" ht="4" customHeight="1">
-      <c r="A277" s="25" t="n"/>
-      <c r="B277" s="25" t="n"/>
-      <c r="C277" s="25" t="n"/>
-      <c r="D277" s="25" t="n"/>
-      <c r="E277" s="25" t="n"/>
-      <c r="F277" s="25" t="n"/>
-      <c r="G277" s="25" t="n"/>
-    </row>
-    <row r="278">
-      <c r="A278" s="15" t="inlineStr">
-        <is>
-          <t>notification</t>
-        </is>
-      </c>
-      <c r="B278" s="16" t="inlineStr">
-        <is>
-          <t>id</t>
-        </is>
-      </c>
-      <c r="C278" s="17" t="inlineStr">
-        <is>
-          <t>bigint</t>
-        </is>
-      </c>
-      <c r="D278" s="18" t="inlineStr">
-        <is>
-          <t>PK</t>
-        </is>
-      </c>
-      <c r="E278" s="19" t="inlineStr"/>
-      <c r="F278" s="20" t="inlineStr">
-        <is>
-          <t>NOT NULL</t>
-        </is>
-      </c>
-      <c r="G278" s="4" t="inlineStr"/>
-    </row>
-    <row r="279">
-      <c r="A279" s="3" t="inlineStr"/>
-      <c r="B279" s="17" t="inlineStr">
-        <is>
-          <t>recipient_user_id</t>
-        </is>
-      </c>
-      <c r="C279" s="17" t="inlineStr">
-        <is>
-          <t>bigint</t>
-        </is>
-      </c>
-      <c r="D279" s="24" t="inlineStr">
-        <is>
-          <t>FK</t>
-        </is>
-      </c>
-      <c r="E279" s="19" t="inlineStr">
-        <is>
-          <t>app_user(id)</t>
-        </is>
-      </c>
-      <c r="F279" s="23" t="inlineStr">
-        <is>
-          <t>NULL</t>
-        </is>
-      </c>
-      <c r="G279" s="4" t="inlineStr"/>
-    </row>
-    <row r="280">
-      <c r="A280" s="3" t="inlineStr"/>
-      <c r="B280" s="17" t="inlineStr">
-        <is>
-          <t>message</t>
-        </is>
-      </c>
-      <c r="C280" s="17" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="D280" s="22" t="inlineStr"/>
-      <c r="E280" s="19" t="inlineStr"/>
-      <c r="F280" s="20" t="inlineStr">
-        <is>
-          <t>NOT NULL</t>
-        </is>
-      </c>
-      <c r="G280" s="4" t="inlineStr"/>
-    </row>
-    <row r="281">
-      <c r="A281" s="3" t="inlineStr"/>
-      <c r="B281" s="17" t="inlineStr">
-        <is>
-          <t>channel</t>
-        </is>
-      </c>
-      <c r="C281" s="21" t="inlineStr">
-        <is>
-          <t>notification_channel</t>
-        </is>
-      </c>
-      <c r="D281" s="22" t="inlineStr"/>
-      <c r="E281" s="19" t="inlineStr"/>
-      <c r="F281" s="20" t="inlineStr">
-        <is>
-          <t>NOT NULL</t>
-        </is>
-      </c>
-      <c r="G281" s="4" t="inlineStr">
-        <is>
-          <t>ENUM: sms/email/push/in_app</t>
-        </is>
-      </c>
-    </row>
-    <row r="282">
-      <c r="A282" s="3" t="inlineStr"/>
-      <c r="B282" s="17" t="inlineStr">
-        <is>
-          <t>escalation_level</t>
-        </is>
-      </c>
-      <c r="C282" s="17" t="inlineStr">
-        <is>
-          <t>smallint</t>
-        </is>
-      </c>
-      <c r="D282" s="22" t="inlineStr"/>
-      <c r="E282" s="19" t="inlineStr"/>
-      <c r="F282" s="23" t="inlineStr">
-        <is>
-          <t>NULL</t>
-        </is>
-      </c>
-      <c r="G282" s="4" t="inlineStr"/>
-    </row>
-    <row r="283">
-      <c r="A283" s="3" t="inlineStr"/>
-      <c r="B283" s="17" t="inlineStr">
-        <is>
-          <t>sent_at</t>
-        </is>
-      </c>
-      <c r="C283" s="21" t="inlineStr">
-        <is>
-          <t>timestamptz</t>
-        </is>
-      </c>
-      <c r="D283" s="22" t="inlineStr"/>
-      <c r="E283" s="19" t="inlineStr"/>
-      <c r="F283" s="23" t="inlineStr">
-        <is>
-          <t>NULL</t>
-        </is>
-      </c>
-      <c r="G283" s="4" t="inlineStr"/>
-    </row>
-    <row r="284">
-      <c r="A284" s="3" t="inlineStr"/>
-      <c r="B284" s="17" t="inlineStr">
-        <is>
-          <t>is_read</t>
-        </is>
-      </c>
-      <c r="C284" s="17" t="inlineStr">
-        <is>
-          <t>boolean</t>
-        </is>
-      </c>
-      <c r="D284" s="22" t="inlineStr"/>
-      <c r="E284" s="19" t="inlineStr"/>
-      <c r="F284" s="20" t="inlineStr">
-        <is>
-          <t>NOT NULL</t>
-        </is>
-      </c>
-      <c r="G284" s="4" t="inlineStr"/>
-    </row>
-    <row r="285">
-      <c r="A285" s="3" t="inlineStr"/>
-      <c r="B285" s="17" t="inlineStr">
-        <is>
-          <t>created_at</t>
-        </is>
-      </c>
-      <c r="C285" s="21" t="inlineStr">
-        <is>
-          <t>timestamptz</t>
-        </is>
-      </c>
-      <c r="D285" s="22" t="inlineStr"/>
-      <c r="E285" s="19" t="inlineStr"/>
-      <c r="F285" s="20" t="inlineStr">
-        <is>
-          <t>NOT NULL</t>
-        </is>
-      </c>
-      <c r="G285" s="4" t="inlineStr"/>
-    </row>
-    <row r="286" ht="4" customHeight="1">
-      <c r="A286" s="25" t="n"/>
-      <c r="B286" s="25" t="n"/>
-      <c r="C286" s="25" t="n"/>
-      <c r="D286" s="25" t="n"/>
-      <c r="E286" s="25" t="n"/>
-      <c r="F286" s="25" t="n"/>
-      <c r="G286" s="25" t="n"/>
-    </row>
-    <row r="287">
-      <c r="A287" s="15" t="inlineStr">
-        <is>
-          <t>report</t>
-        </is>
-      </c>
-      <c r="B287" s="16" t="inlineStr">
-        <is>
-          <t>id</t>
-        </is>
-      </c>
-      <c r="C287" s="17" t="inlineStr">
-        <is>
-          <t>bigint</t>
-        </is>
-      </c>
-      <c r="D287" s="18" t="inlineStr">
-        <is>
-          <t>PK</t>
-        </is>
-      </c>
-      <c r="E287" s="19" t="inlineStr"/>
-      <c r="F287" s="20" t="inlineStr">
-        <is>
-          <t>NOT NULL</t>
-        </is>
-      </c>
-      <c r="G287" s="4" t="inlineStr"/>
-    </row>
-    <row r="288">
-      <c r="A288" s="3" t="inlineStr"/>
-      <c r="B288" s="17" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="C288" s="21" t="inlineStr">
-        <is>
-          <t>varchar(160)</t>
-        </is>
-      </c>
-      <c r="D288" s="22" t="inlineStr"/>
-      <c r="E288" s="19" t="inlineStr"/>
-      <c r="F288" s="23" t="inlineStr">
-        <is>
-          <t>NULL</t>
-        </is>
-      </c>
-      <c r="G288" s="4" t="inlineStr"/>
-    </row>
-    <row r="289">
-      <c r="A289" s="3" t="inlineStr"/>
-      <c r="B289" s="17" t="inlineStr">
-        <is>
-          <t>template_ref</t>
-        </is>
-      </c>
-      <c r="C289" s="21" t="inlineStr">
-        <is>
-          <t>varchar(120)</t>
-        </is>
-      </c>
-      <c r="D289" s="22" t="inlineStr"/>
-      <c r="E289" s="19" t="inlineStr"/>
-      <c r="F289" s="23" t="inlineStr">
-        <is>
-          <t>NULL</t>
-        </is>
-      </c>
-      <c r="G289" s="4" t="inlineStr"/>
-    </row>
-    <row r="290">
-      <c r="A290" s="3" t="inlineStr"/>
-      <c r="B290" s="17" t="inlineStr">
-        <is>
-          <t>created_at</t>
-        </is>
-      </c>
-      <c r="C290" s="21" t="inlineStr">
-        <is>
-          <t>timestamptz</t>
-        </is>
-      </c>
-      <c r="D290" s="22" t="inlineStr"/>
-      <c r="E290" s="19" t="inlineStr"/>
-      <c r="F290" s="23" t="inlineStr">
-        <is>
-          <t>NULL</t>
-        </is>
-      </c>
-      <c r="G290" s="4" t="inlineStr"/>
-    </row>
-    <row r="291" ht="4" customHeight="1">
-      <c r="A291" s="25" t="n"/>
-      <c r="B291" s="25" t="n"/>
-      <c r="C291" s="25" t="n"/>
-      <c r="D291" s="25" t="n"/>
-      <c r="E291" s="25" t="n"/>
-      <c r="F291" s="25" t="n"/>
-      <c r="G291" s="25" t="n"/>
-    </row>
-    <row r="292">
-      <c r="A292" s="15" t="inlineStr">
-        <is>
-          <t>evaluation</t>
-        </is>
-      </c>
-      <c r="B292" s="16" t="inlineStr">
-        <is>
-          <t>id</t>
-        </is>
-      </c>
-      <c r="C292" s="17" t="inlineStr">
-        <is>
-          <t>bigint</t>
-        </is>
-      </c>
-      <c r="D292" s="18" t="inlineStr">
-        <is>
-          <t>PK</t>
-        </is>
-      </c>
-      <c r="E292" s="19" t="inlineStr"/>
-      <c r="F292" s="20" t="inlineStr">
-        <is>
-          <t>NOT NULL</t>
-        </is>
-      </c>
-      <c r="G292" s="4" t="inlineStr"/>
-    </row>
-    <row r="293">
-      <c r="A293" s="3" t="inlineStr"/>
-      <c r="B293" s="17" t="inlineStr">
-        <is>
-          <t>subject_type</t>
-        </is>
-      </c>
-      <c r="C293" s="21" t="inlineStr">
-        <is>
-          <t>varchar(40)</t>
-        </is>
-      </c>
-      <c r="D293" s="22" t="inlineStr"/>
-      <c r="E293" s="19" t="inlineStr"/>
-      <c r="F293" s="23" t="inlineStr">
-        <is>
-          <t>NULL</t>
-        </is>
-      </c>
-      <c r="G293" s="4" t="inlineStr">
-        <is>
-          <t>student/trainer/group</t>
-        </is>
-      </c>
-    </row>
-    <row r="294">
-      <c r="A294" s="3" t="inlineStr"/>
-      <c r="B294" s="17" t="inlineStr">
-        <is>
-          <t>subject_id</t>
-        </is>
-      </c>
-      <c r="C294" s="17" t="inlineStr">
-        <is>
-          <t>bigint</t>
-        </is>
-      </c>
-      <c r="D294" s="22" t="inlineStr"/>
-      <c r="E294" s="19" t="inlineStr"/>
-      <c r="F294" s="23" t="inlineStr">
-        <is>
-          <t>NULL</t>
-        </is>
-      </c>
-      <c r="G294" s="4" t="inlineStr">
-        <is>
-          <t>Polymorphic ref</t>
-        </is>
-      </c>
-    </row>
-    <row r="295">
-      <c r="A295" s="3" t="inlineStr"/>
-      <c r="B295" s="17" t="inlineStr">
-        <is>
-          <t>score</t>
-        </is>
-      </c>
-      <c r="C295" s="21" t="inlineStr">
-        <is>
-          <t>numeric(5,2)</t>
-        </is>
-      </c>
-      <c r="D295" s="22" t="inlineStr"/>
-      <c r="E295" s="19" t="inlineStr"/>
-      <c r="F295" s="23" t="inlineStr">
-        <is>
-          <t>NULL</t>
-        </is>
-      </c>
-      <c r="G295" s="4" t="inlineStr"/>
-    </row>
-    <row r="296">
-      <c r="A296" s="3" t="inlineStr"/>
-      <c r="B296" s="17" t="inlineStr">
-        <is>
-          <t>created_at</t>
-        </is>
-      </c>
-      <c r="C296" s="21" t="inlineStr">
-        <is>
-          <t>timestamptz</t>
-        </is>
-      </c>
-      <c r="D296" s="22" t="inlineStr"/>
-      <c r="E296" s="19" t="inlineStr"/>
-      <c r="F296" s="23" t="inlineStr">
-        <is>
-          <t>NULL</t>
-        </is>
-      </c>
-      <c r="G296" s="4" t="inlineStr"/>
-    </row>
-    <row r="297" ht="4" customHeight="1">
-      <c r="A297" s="25" t="n"/>
-      <c r="B297" s="25" t="n"/>
-      <c r="C297" s="25" t="n"/>
-      <c r="D297" s="25" t="n"/>
-      <c r="E297" s="25" t="n"/>
-      <c r="F297" s="25" t="n"/>
-      <c r="G297" s="25" t="n"/>
-    </row>
-    <row r="298">
-      <c r="A298" s="15" t="inlineStr">
-        <is>
-          <t>knowledge_article</t>
-        </is>
-      </c>
-      <c r="B298" s="16" t="inlineStr">
-        <is>
-          <t>id</t>
-        </is>
-      </c>
-      <c r="C298" s="17" t="inlineStr">
-        <is>
-          <t>bigint</t>
-        </is>
-      </c>
-      <c r="D298" s="18" t="inlineStr">
-        <is>
-          <t>PK</t>
-        </is>
-      </c>
-      <c r="E298" s="19" t="inlineStr"/>
-      <c r="F298" s="20" t="inlineStr">
-        <is>
-          <t>NOT NULL</t>
-        </is>
-      </c>
-      <c r="G298" s="4" t="inlineStr"/>
-    </row>
-    <row r="299">
-      <c r="A299" s="3" t="inlineStr"/>
-      <c r="B299" s="17" t="inlineStr">
-        <is>
-          <t>title</t>
-        </is>
-      </c>
-      <c r="C299" s="21" t="inlineStr">
-        <is>
-          <t>varchar(160)</t>
-        </is>
-      </c>
-      <c r="D299" s="22" t="inlineStr"/>
-      <c r="E299" s="19" t="inlineStr"/>
-      <c r="F299" s="23" t="inlineStr">
-        <is>
-          <t>NULL</t>
-        </is>
-      </c>
-      <c r="G299" s="4" t="inlineStr"/>
-    </row>
-    <row r="300">
-      <c r="A300" s="3" t="inlineStr"/>
-      <c r="B300" s="17" t="inlineStr">
-        <is>
-          <t>body</t>
-        </is>
-      </c>
-      <c r="C300" s="17" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="D300" s="22" t="inlineStr"/>
-      <c r="E300" s="19" t="inlineStr"/>
-      <c r="F300" s="23" t="inlineStr">
-        <is>
-          <t>NULL</t>
-        </is>
-      </c>
-      <c r="G300" s="4" t="inlineStr"/>
-    </row>
-    <row r="301">
-      <c r="A301" s="3" t="inlineStr"/>
-      <c r="B301" s="17" t="inlineStr">
-        <is>
-          <t>created_at</t>
-        </is>
-      </c>
-      <c r="C301" s="21" t="inlineStr">
-        <is>
-          <t>timestamptz</t>
-        </is>
-      </c>
-      <c r="D301" s="22" t="inlineStr"/>
-      <c r="E301" s="19" t="inlineStr"/>
-      <c r="F301" s="23" t="inlineStr">
-        <is>
-          <t>NULL</t>
-        </is>
-      </c>
-      <c r="G301" s="4" t="inlineStr"/>
-    </row>
-    <row r="302" ht="4" customHeight="1">
-      <c r="A302" s="25" t="n"/>
-      <c r="B302" s="25" t="n"/>
-      <c r="C302" s="25" t="n"/>
-      <c r="D302" s="25" t="n"/>
-      <c r="E302" s="25" t="n"/>
-      <c r="F302" s="25" t="n"/>
-      <c r="G302" s="25" t="n"/>
-    </row>
-    <row r="303">
-      <c r="A303" s="15" t="inlineStr">
-        <is>
-          <t>module_progress</t>
-        </is>
-      </c>
-      <c r="B303" s="17" t="inlineStr">
-        <is>
-          <t>student_id</t>
-        </is>
-      </c>
-      <c r="C303" s="17" t="inlineStr">
-        <is>
-          <t>bigint</t>
-        </is>
-      </c>
-      <c r="D303" s="24" t="inlineStr">
-        <is>
-          <t>FK</t>
-        </is>
-      </c>
-      <c r="E303" s="19" t="inlineStr">
-        <is>
-          <t>student(id)</t>
-        </is>
-      </c>
-      <c r="F303" s="20" t="inlineStr">
-        <is>
-          <t>NOT NULL</t>
-        </is>
-      </c>
-      <c r="G303" s="4" t="inlineStr">
-        <is>
-          <t>Part of composite key</t>
-        </is>
-      </c>
-    </row>
-    <row r="304">
-      <c r="A304" s="3" t="inlineStr"/>
-      <c r="B304" s="17" t="inlineStr">
-        <is>
-          <t>module_id</t>
-        </is>
-      </c>
-      <c r="C304" s="17" t="inlineStr">
-        <is>
-          <t>bigint</t>
-        </is>
-      </c>
-      <c r="D304" s="24" t="inlineStr">
-        <is>
-          <t>FK</t>
-        </is>
-      </c>
-      <c r="E304" s="19" t="inlineStr">
-        <is>
-          <t>module(id)</t>
-        </is>
-      </c>
-      <c r="F304" s="20" t="inlineStr">
-        <is>
-          <t>NOT NULL</t>
-        </is>
-      </c>
-      <c r="G304" s="4" t="inlineStr">
-        <is>
-          <t>Part of composite key</t>
-        </is>
-      </c>
-    </row>
-    <row r="305">
-      <c r="A305" s="3" t="inlineStr"/>
-      <c r="B305" s="17" t="inlineStr">
-        <is>
-          <t>completed_lectures</t>
-        </is>
-      </c>
-      <c r="C305" s="17" t="inlineStr">
-        <is>
-          <t>integer</t>
-        </is>
-      </c>
-      <c r="D305" s="22" t="inlineStr"/>
-      <c r="E305" s="19" t="inlineStr"/>
-      <c r="F305" s="20" t="inlineStr">
-        <is>
-          <t>NOT NULL</t>
-        </is>
-      </c>
-      <c r="G305" s="4" t="inlineStr">
+      <c r="G262" s="4" t="inlineStr">
         <is>
           <t>Computed</t>
         </is>
       </c>
     </row>
-    <row r="306">
-      <c r="A306" s="3" t="inlineStr"/>
-      <c r="B306" s="17" t="inlineStr">
-        <is>
-          <t>total_lectures</t>
-        </is>
-      </c>
-      <c r="C306" s="17" t="inlineStr">
-        <is>
-          <t>integer</t>
-        </is>
-      </c>
-      <c r="D306" s="22" t="inlineStr"/>
-      <c r="E306" s="19" t="inlineStr"/>
-      <c r="F306" s="20" t="inlineStr">
-        <is>
-          <t>NOT NULL</t>
-        </is>
-      </c>
-      <c r="G306" s="4" t="inlineStr">
-        <is>
-          <t>Computed</t>
-        </is>
-      </c>
-    </row>
-    <row r="307">
-      <c r="A307" s="3" t="inlineStr"/>
-      <c r="B307" s="17" t="inlineStr">
-        <is>
-          <t>progress_pct</t>
-        </is>
-      </c>
-      <c r="C307" s="21" t="inlineStr">
-        <is>
-          <t>numeric(5,2)</t>
-        </is>
-      </c>
-      <c r="D307" s="22" t="inlineStr"/>
-      <c r="E307" s="19" t="inlineStr"/>
-      <c r="F307" s="20" t="inlineStr">
-        <is>
-          <t>NOT NULL</t>
-        </is>
-      </c>
-      <c r="G307" s="4" t="inlineStr">
-        <is>
-          <t>Computed</t>
-        </is>
-      </c>
-    </row>
-    <row r="308" ht="4" customHeight="1">
-      <c r="A308" s="25" t="n"/>
-      <c r="B308" s="25" t="n"/>
-      <c r="C308" s="25" t="n"/>
-      <c r="D308" s="25" t="n"/>
-      <c r="E308" s="25" t="n"/>
-      <c r="F308" s="25" t="n"/>
-      <c r="G308" s="25" t="n"/>
-    </row>
-    <row r="309">
-      <c r="A309" s="15" t="inlineStr">
-        <is>
-          <t>debt</t>
-        </is>
-      </c>
-      <c r="B309" s="17" t="inlineStr">
-        <is>
-          <t>student_id</t>
-        </is>
-      </c>
-      <c r="C309" s="17" t="inlineStr">
-        <is>
-          <t>bigint</t>
-        </is>
-      </c>
-      <c r="D309" s="24" t="inlineStr">
-        <is>
-          <t>FK</t>
-        </is>
-      </c>
-      <c r="E309" s="19" t="inlineStr">
-        <is>
-          <t>student(id)</t>
-        </is>
-      </c>
-      <c r="F309" s="20" t="inlineStr">
-        <is>
-          <t>NOT NULL</t>
-        </is>
-      </c>
-      <c r="G309" s="4" t="inlineStr">
-        <is>
-          <t>Key</t>
-        </is>
-      </c>
-    </row>
-    <row r="310">
-      <c r="A310" s="3" t="inlineStr"/>
-      <c r="B310" s="17" t="inlineStr">
-        <is>
-          <t>outstanding_amount</t>
-        </is>
-      </c>
-      <c r="C310" s="21" t="inlineStr">
-        <is>
-          <t>numeric(10,2)</t>
-        </is>
-      </c>
-      <c r="D310" s="22" t="inlineStr"/>
-      <c r="E310" s="19" t="inlineStr"/>
-      <c r="F310" s="20" t="inlineStr">
-        <is>
-          <t>NOT NULL</t>
-        </is>
-      </c>
-      <c r="G310" s="4" t="inlineStr">
-        <is>
-          <t>Computed</t>
-        </is>
-      </c>
-    </row>
-    <row r="311">
-      <c r="A311" s="3" t="inlineStr"/>
-      <c r="B311" s="17" t="inlineStr">
-        <is>
-          <t>overdue_days</t>
-        </is>
-      </c>
-      <c r="C311" s="17" t="inlineStr">
-        <is>
-          <t>integer</t>
-        </is>
-      </c>
-      <c r="D311" s="22" t="inlineStr"/>
-      <c r="E311" s="19" t="inlineStr"/>
-      <c r="F311" s="23" t="inlineStr">
-        <is>
-          <t>NULL</t>
-        </is>
-      </c>
-      <c r="G311" s="4" t="inlineStr">
-        <is>
-          <t>Computed</t>
-        </is>
-      </c>
-    </row>
-    <row r="312" ht="4" customHeight="1">
-      <c r="A312" s="25" t="n"/>
-      <c r="B312" s="25" t="n"/>
-      <c r="C312" s="25" t="n"/>
-      <c r="D312" s="25" t="n"/>
-      <c r="E312" s="25" t="n"/>
-      <c r="F312" s="25" t="n"/>
-      <c r="G312" s="25" t="n"/>
+    <row r="263" ht="4" customHeight="1">
+      <c r="A263" s="25" t="n"/>
+      <c r="B263" s="25" t="n"/>
+      <c r="C263" s="25" t="n"/>
+      <c r="D263" s="25" t="n"/>
+      <c r="E263" s="25" t="n"/>
+      <c r="F263" s="25" t="n"/>
+      <c r="G263" s="25" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G312"/>
+  <autoFilter ref="A1:G263"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -9229,7 +7938,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G71"/>
+  <dimension ref="A1:G64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -11209,7 +9918,7 @@
       </c>
       <c r="B57" s="11" t="inlineStr">
         <is>
-          <t>payment</t>
+          <t>subscription</t>
         </is>
       </c>
       <c r="C57" s="13" t="inlineStr">
@@ -11234,7 +9943,7 @@
       </c>
       <c r="G57" s="12" t="inlineStr">
         <is>
-          <t>payment → student</t>
+          <t>subscription → student</t>
         </is>
       </c>
     </row>
@@ -11244,17 +9953,17 @@
       </c>
       <c r="B58" s="7" t="inlineStr">
         <is>
-          <t>payment</t>
+          <t>subscription</t>
         </is>
       </c>
       <c r="C58" s="9" t="inlineStr">
         <is>
-          <t>semester_id</t>
+          <t>parent_id</t>
         </is>
       </c>
       <c r="D58" s="27" t="inlineStr">
         <is>
-          <t>semester(id)</t>
+          <t>parent(id)</t>
         </is>
       </c>
       <c r="E58" s="6" t="inlineStr">
@@ -11269,7 +9978,7 @@
       </c>
       <c r="G58" s="8" t="inlineStr">
         <is>
-          <t>payment → semester</t>
+          <t>subscription → parent</t>
         </is>
       </c>
     </row>
@@ -11279,7 +9988,7 @@
       </c>
       <c r="B59" s="11" t="inlineStr">
         <is>
-          <t>subscription</t>
+          <t>module_progress</t>
         </is>
       </c>
       <c r="C59" s="13" t="inlineStr">
@@ -11304,7 +10013,7 @@
       </c>
       <c r="G59" s="12" t="inlineStr">
         <is>
-          <t>subscription → student</t>
+          <t>Part of composite key</t>
         </is>
       </c>
     </row>
@@ -11314,17 +10023,17 @@
       </c>
       <c r="B60" s="7" t="inlineStr">
         <is>
-          <t>subscription</t>
+          <t>module_progress</t>
         </is>
       </c>
       <c r="C60" s="9" t="inlineStr">
         <is>
-          <t>parent_id</t>
+          <t>module_id</t>
         </is>
       </c>
       <c r="D60" s="27" t="inlineStr">
         <is>
-          <t>parent(id)</t>
+          <t>module(id)</t>
         </is>
       </c>
       <c r="E60" s="6" t="inlineStr">
@@ -11334,335 +10043,90 @@
       </c>
       <c r="F60" s="28" t="inlineStr">
         <is>
-          <t>SET NULL</t>
+          <t>RESTRICT</t>
         </is>
       </c>
       <c r="G60" s="8" t="inlineStr">
         <is>
-          <t>subscription → parent</t>
+          <t>Part of composite key</t>
         </is>
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="10" t="n">
-        <v>60</v>
-      </c>
-      <c r="B61" s="11" t="inlineStr">
-        <is>
-          <t>document</t>
-        </is>
-      </c>
-      <c r="C61" s="13" t="inlineStr">
-        <is>
-          <t>owner_user_id</t>
-        </is>
-      </c>
-      <c r="D61" s="29" t="inlineStr">
-        <is>
-          <t>app_user(id)</t>
-        </is>
-      </c>
-      <c r="E61" s="10" t="inlineStr">
-        <is>
-          <t>N:1</t>
-        </is>
-      </c>
-      <c r="F61" s="30" t="inlineStr">
-        <is>
-          <t>SET NULL</t>
-        </is>
-      </c>
-      <c r="G61" s="12" t="inlineStr">
-        <is>
-          <t>document → app_user</t>
+      <c r="B61" s="31" t="inlineStr">
+        <is>
+          <t>— Many-to-many resolutions —</t>
         </is>
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="6" t="n">
-        <v>61</v>
-      </c>
-      <c r="B62" s="7" t="inlineStr">
-        <is>
-          <t>document</t>
-        </is>
-      </c>
-      <c r="C62" s="9" t="inlineStr">
-        <is>
-          <t>student_id</t>
-        </is>
-      </c>
-      <c r="D62" s="27" t="inlineStr">
-        <is>
-          <t>student(id)</t>
-        </is>
-      </c>
-      <c r="E62" s="6" t="inlineStr">
-        <is>
-          <t>N:1</t>
-        </is>
-      </c>
-      <c r="F62" s="28" t="inlineStr">
-        <is>
-          <t>SET NULL</t>
-        </is>
-      </c>
-      <c r="G62" s="8" t="inlineStr">
-        <is>
-          <t>document → student</t>
+      <c r="B62" s="3" t="inlineStr">
+        <is>
+          <t>student_parent</t>
+        </is>
+      </c>
+      <c r="D62" s="19" t="inlineStr">
+        <is>
+          <t>student ↔ parent</t>
+        </is>
+      </c>
+      <c r="E62" s="22" t="inlineStr">
+        <is>
+          <t>M:N</t>
+        </is>
+      </c>
+      <c r="G62" s="4" t="inlineStr">
+        <is>
+          <t>via student_parent</t>
         </is>
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="10" t="n">
-        <v>62</v>
-      </c>
-      <c r="B63" s="11" t="inlineStr">
-        <is>
-          <t>document</t>
-        </is>
-      </c>
-      <c r="C63" s="13" t="inlineStr">
-        <is>
-          <t>uploaded_by</t>
-        </is>
-      </c>
-      <c r="D63" s="29" t="inlineStr">
-        <is>
-          <t>app_user(id)</t>
-        </is>
-      </c>
-      <c r="E63" s="10" t="inlineStr">
-        <is>
-          <t>N:1</t>
-        </is>
-      </c>
-      <c r="F63" s="30" t="inlineStr">
-        <is>
-          <t>SET NULL</t>
-        </is>
-      </c>
-      <c r="G63" s="12" t="inlineStr">
-        <is>
-          <t>document → app_user</t>
+      <c r="B63" s="3" t="inlineStr">
+        <is>
+          <t>group_membership</t>
+        </is>
+      </c>
+      <c r="D63" s="19" t="inlineStr">
+        <is>
+          <t>student ↔ study_group</t>
+        </is>
+      </c>
+      <c r="E63" s="22" t="inlineStr">
+        <is>
+          <t>M:N</t>
+        </is>
+      </c>
+      <c r="G63" s="4" t="inlineStr">
+        <is>
+          <t>via group_membership</t>
         </is>
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="6" t="n">
-        <v>63</v>
-      </c>
-      <c r="B64" s="7" t="inlineStr">
-        <is>
-          <t>notification</t>
-        </is>
-      </c>
-      <c r="C64" s="9" t="inlineStr">
-        <is>
-          <t>recipient_user_id</t>
-        </is>
-      </c>
-      <c r="D64" s="27" t="inlineStr">
-        <is>
-          <t>app_user(id)</t>
-        </is>
-      </c>
-      <c r="E64" s="6" t="inlineStr">
-        <is>
-          <t>N:1</t>
-        </is>
-      </c>
-      <c r="F64" s="28" t="inlineStr">
-        <is>
-          <t>SET NULL</t>
-        </is>
-      </c>
-      <c r="G64" s="8" t="inlineStr">
-        <is>
-          <t>notification → app_user</t>
-        </is>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" s="10" t="n">
-        <v>64</v>
-      </c>
-      <c r="B65" s="11" t="inlineStr">
-        <is>
-          <t>module_progress</t>
-        </is>
-      </c>
-      <c r="C65" s="13" t="inlineStr">
-        <is>
-          <t>student_id</t>
-        </is>
-      </c>
-      <c r="D65" s="29" t="inlineStr">
-        <is>
-          <t>student(id)</t>
-        </is>
-      </c>
-      <c r="E65" s="10" t="inlineStr">
-        <is>
-          <t>N:1</t>
-        </is>
-      </c>
-      <c r="F65" s="30" t="inlineStr">
-        <is>
-          <t>RESTRICT</t>
-        </is>
-      </c>
-      <c r="G65" s="12" t="inlineStr">
-        <is>
-          <t>Part of composite key</t>
-        </is>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" s="6" t="n">
-        <v>65</v>
-      </c>
-      <c r="B66" s="7" t="inlineStr">
-        <is>
-          <t>module_progress</t>
-        </is>
-      </c>
-      <c r="C66" s="9" t="inlineStr">
-        <is>
-          <t>module_id</t>
-        </is>
-      </c>
-      <c r="D66" s="27" t="inlineStr">
-        <is>
-          <t>module(id)</t>
-        </is>
-      </c>
-      <c r="E66" s="6" t="inlineStr">
-        <is>
-          <t>N:1</t>
-        </is>
-      </c>
-      <c r="F66" s="28" t="inlineStr">
-        <is>
-          <t>RESTRICT</t>
-        </is>
-      </c>
-      <c r="G66" s="8" t="inlineStr">
-        <is>
-          <t>Part of composite key</t>
-        </is>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" s="10" t="n">
-        <v>66</v>
-      </c>
-      <c r="B67" s="11" t="inlineStr">
-        <is>
-          <t>debt</t>
-        </is>
-      </c>
-      <c r="C67" s="13" t="inlineStr">
-        <is>
-          <t>student_id</t>
-        </is>
-      </c>
-      <c r="D67" s="29" t="inlineStr">
-        <is>
-          <t>student(id)</t>
-        </is>
-      </c>
-      <c r="E67" s="10" t="inlineStr">
-        <is>
-          <t>N:1</t>
-        </is>
-      </c>
-      <c r="F67" s="30" t="inlineStr">
-        <is>
-          <t>RESTRICT</t>
-        </is>
-      </c>
-      <c r="G67" s="12" t="inlineStr">
-        <is>
-          <t>Key</t>
-        </is>
-      </c>
-    </row>
-    <row r="68">
-      <c r="B68" s="31" t="inlineStr">
-        <is>
-          <t>— Many-to-many resolutions —</t>
-        </is>
-      </c>
-    </row>
-    <row r="69">
-      <c r="B69" s="3" t="inlineStr">
-        <is>
-          <t>student_parent</t>
-        </is>
-      </c>
-      <c r="D69" s="19" t="inlineStr">
-        <is>
-          <t>student ↔ parent</t>
-        </is>
-      </c>
-      <c r="E69" s="22" t="inlineStr">
+      <c r="B64" s="3" t="inlineStr">
+        <is>
+          <t>project_participation</t>
+        </is>
+      </c>
+      <c r="D64" s="19" t="inlineStr">
+        <is>
+          <t>student ↔ project</t>
+        </is>
+      </c>
+      <c r="E64" s="22" t="inlineStr">
         <is>
           <t>M:N</t>
         </is>
       </c>
-      <c r="G69" s="4" t="inlineStr">
-        <is>
-          <t>via student_parent</t>
-        </is>
-      </c>
-    </row>
-    <row r="70">
-      <c r="B70" s="3" t="inlineStr">
-        <is>
-          <t>group_membership</t>
-        </is>
-      </c>
-      <c r="D70" s="19" t="inlineStr">
-        <is>
-          <t>student ↔ study_group</t>
-        </is>
-      </c>
-      <c r="E70" s="22" t="inlineStr">
-        <is>
-          <t>M:N</t>
-        </is>
-      </c>
-      <c r="G70" s="4" t="inlineStr">
-        <is>
-          <t>via group_membership</t>
-        </is>
-      </c>
-    </row>
-    <row r="71">
-      <c r="B71" s="3" t="inlineStr">
-        <is>
-          <t>project_participation</t>
-        </is>
-      </c>
-      <c r="D71" s="19" t="inlineStr">
-        <is>
-          <t>student ↔ project</t>
-        </is>
-      </c>
-      <c r="E71" s="22" t="inlineStr">
-        <is>
-          <t>M:N</t>
-        </is>
-      </c>
-      <c r="G71" s="4" t="inlineStr">
+      <c r="G64" s="4" t="inlineStr">
         <is>
           <t>via project_participation</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G67"/>
+  <autoFilter ref="A1:G60"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -11673,7 +10137,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F39"/>
+  <dimension ref="A1:F32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -12140,17 +10604,17 @@
       </c>
       <c r="B15" s="12" t="inlineStr">
         <is>
-          <t>Module Templates</t>
+          <t>Module Templates › category (mAddTemplate)</t>
         </is>
       </c>
       <c r="C15" s="12" t="inlineStr">
         <is>
-          <t>Module Templates grid + template detail</t>
+          <t>Module Templates grid → category list → template detail</t>
         </is>
       </c>
       <c r="D15" s="12" t="inlineStr">
         <is>
-          <t>Template detail</t>
+          <t>Template detail / Edit Lecture</t>
         </is>
       </c>
       <c r="E15" s="12" t="inlineStr">
@@ -12204,7 +10668,7 @@
       </c>
       <c r="B17" s="12" t="inlineStr">
         <is>
-          <t>Learning Modules (mAddModule)</t>
+          <t>Learning Modules › instantiate template (mAddModule)</t>
         </is>
       </c>
       <c r="C17" s="12" t="inlineStr">
@@ -12214,7 +10678,7 @@
       </c>
       <c r="D17" s="12" t="inlineStr">
         <is>
-          <t>Module detail</t>
+          <t>Module detail / Edit Lecture</t>
         </is>
       </c>
       <c r="E17" s="12" t="inlineStr">
@@ -12583,22 +11047,22 @@
     <row r="29">
       <c r="A29" s="11" t="inlineStr">
         <is>
-          <t>payment</t>
+          <t>subscription</t>
         </is>
       </c>
       <c r="B29" s="12" t="inlineStr">
         <is>
-          <t>Fina integration (auto) + manual entry</t>
+          <t>Parent portal (activate)</t>
         </is>
       </c>
       <c r="C29" s="12" t="inlineStr">
         <is>
-          <t>Payments / Finance</t>
+          <t>Parent / Admin finance</t>
         </is>
       </c>
       <c r="D29" s="12" t="inlineStr">
         <is>
-          <t>Allocate unallocated</t>
+          <t>Activate / cancel</t>
         </is>
       </c>
       <c r="E29" s="12" t="inlineStr">
@@ -12608,280 +11072,56 @@
       </c>
       <c r="F29" s="12" t="inlineStr">
         <is>
-          <t>CRU (create mostly external)</t>
+          <t>CRU</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="7" t="inlineStr">
-        <is>
-          <t>subscription</t>
-        </is>
-      </c>
-      <c r="B30" s="8" t="inlineStr">
-        <is>
-          <t>Parent portal (activate)</t>
-        </is>
-      </c>
-      <c r="C30" s="8" t="inlineStr">
-        <is>
-          <t>Parent / Admin finance</t>
-        </is>
-      </c>
-      <c r="D30" s="8" t="inlineStr">
-        <is>
-          <t>Activate / cancel</t>
-        </is>
-      </c>
-      <c r="E30" s="8" t="inlineStr">
+      <c r="A30" s="32" t="inlineStr">
+        <is>
+          <t>module_progress</t>
+        </is>
+      </c>
+      <c r="B30" s="33" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F30" s="8" t="inlineStr">
-        <is>
-          <t>CRU</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="11" t="inlineStr">
-        <is>
-          <t>document</t>
-        </is>
-      </c>
-      <c r="B31" s="12" t="inlineStr">
-        <is>
-          <t>Documents (mAddDocument)</t>
-        </is>
-      </c>
-      <c r="C31" s="12" t="inlineStr">
-        <is>
-          <t>Documents list</t>
-        </is>
-      </c>
-      <c r="D31" s="12" t="inlineStr">
+      <c r="C30" s="33" t="inlineStr">
+        <is>
+          <t>Student profile progress; dashboards</t>
+        </is>
+      </c>
+      <c r="D30" s="33" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E31" s="12" t="inlineStr">
-        <is>
-          <t>Delete</t>
-        </is>
-      </c>
-      <c r="F31" s="12" t="inlineStr">
-        <is>
-          <t>CRD</t>
+      <c r="E30" s="33" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F30" s="34" t="inlineStr">
+        <is>
+          <t>NONE — derived VIEW (no id; read-only)</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="7" t="inlineStr">
-        <is>
-          <t>notification</t>
-        </is>
-      </c>
-      <c r="B32" s="8" t="inlineStr">
-        <is>
-          <t>System-generated (auto rules)</t>
-        </is>
-      </c>
-      <c r="C32" s="8" t="inlineStr">
-        <is>
-          <t>Notifications screen</t>
-        </is>
-      </c>
-      <c r="D32" s="8" t="inlineStr">
-        <is>
-          <t>Mark read / settings</t>
-        </is>
-      </c>
-      <c r="E32" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F32" s="8" t="inlineStr">
-        <is>
-          <t>RU (create is system, not manual)</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="32" t="inlineStr">
-        <is>
-          <t>report</t>
-        </is>
-      </c>
-      <c r="B33" s="33" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C33" s="33" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D33" s="33" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E33" s="33" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F33" s="34" t="inlineStr">
-        <is>
-          <t>NONE — 'Coming soon', no CRUD point yet</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="32" t="inlineStr">
-        <is>
-          <t>evaluation</t>
-        </is>
-      </c>
-      <c r="B34" s="33" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C34" s="33" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D34" s="33" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E34" s="33" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F34" s="34" t="inlineStr">
-        <is>
-          <t>NONE — 'Coming soon', no CRUD point yet</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="32" t="inlineStr">
-        <is>
-          <t>knowledge_article</t>
-        </is>
-      </c>
-      <c r="B35" s="33" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C35" s="33" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D35" s="33" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E35" s="33" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F35" s="34" t="inlineStr">
-        <is>
-          <t>NONE — 'Coming soon', no CRUD point yet</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="32" t="inlineStr">
-        <is>
-          <t>module_progress</t>
-        </is>
-      </c>
-      <c r="B36" s="33" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C36" s="33" t="inlineStr">
-        <is>
-          <t>Student profile progress; dashboards</t>
-        </is>
-      </c>
-      <c r="D36" s="33" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E36" s="33" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F36" s="34" t="inlineStr">
-        <is>
-          <t>NONE — derived VIEW (no id; read-only)</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="32" t="inlineStr">
-        <is>
-          <t>debt</t>
-        </is>
-      </c>
-      <c r="B37" s="33" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C37" s="33" t="inlineStr">
-        <is>
-          <t>Finance › Debts</t>
-        </is>
-      </c>
-      <c r="D37" s="33" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E37" s="33" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F37" s="34" t="inlineStr">
-        <is>
-          <t>NONE — derived VIEW (read-only)</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="31" t="inlineStr">
+      <c r="A32" s="31" t="inlineStr">
         <is>
           <t>Entities with NO CRUD point:</t>
         </is>
       </c>
-      <c r="B39" s="4" t="inlineStr">
-        <is>
-          <t>program, report, evaluation, knowledge_article, module_progress, debt</t>
+      <c r="B32" s="4" t="inlineStr">
+        <is>
+          <t>program, module_progress</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F37"/>
+  <autoFilter ref="A1:F30"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -12892,7 +11132,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:C13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -13073,90 +11313,56 @@
     <row r="11">
       <c r="A11" s="37" t="inlineStr">
         <is>
-          <t>payment_status</t>
+          <t>intake_season</t>
         </is>
       </c>
       <c r="B11" s="12" t="inlineStr">
         <is>
-          <t>paid, pending, unallocated, overdue</t>
+          <t>spring, autumn</t>
         </is>
       </c>
       <c r="C11" s="38" t="inlineStr">
         <is>
-          <t>payment.status</t>
+          <t>intake.season</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="35" t="inlineStr">
         <is>
-          <t>intake_season</t>
+          <t>relationship_type</t>
         </is>
       </c>
       <c r="B12" s="8" t="inlineStr">
         <is>
-          <t>spring, autumn</t>
+          <t>mother, father, guardian, other</t>
         </is>
       </c>
       <c r="C12" s="36" t="inlineStr">
         <is>
-          <t>intake.season</t>
+          <t>student_parent.relationship</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="37" t="inlineStr">
         <is>
-          <t>relationship_type</t>
+          <t>project_result</t>
         </is>
       </c>
       <c r="B13" s="12" t="inlineStr">
         <is>
-          <t>mother, father, guardian, other</t>
+          <t>participated, won, completed</t>
         </is>
       </c>
       <c r="C13" s="38" t="inlineStr">
         <is>
-          <t>student_parent.relationship</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="35" t="inlineStr">
-        <is>
-          <t>project_result</t>
-        </is>
-      </c>
-      <c r="B14" s="8" t="inlineStr">
-        <is>
-          <t>participated, won, completed</t>
-        </is>
-      </c>
-      <c r="C14" s="36" t="inlineStr">
-        <is>
           <t>project_participation.result</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="37" t="inlineStr">
-        <is>
-          <t>notification_channel</t>
-        </is>
-      </c>
-      <c r="B15" s="12" t="inlineStr">
-        <is>
-          <t>sms, email, push, in_app</t>
-        </is>
-      </c>
-      <c r="C15" s="38" t="inlineStr">
-        <is>
-          <t>notification.channel</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:C15"/>
+  <autoFilter ref="A1:C13"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
RBAC: Branch Manager is a locked system group; custom groups use Admin UI
- admin Users & Groups: Branch Manager moved into the 🔒 System · locked
  set (its own interface, manager.html); the four system groups are
  Students/Parents/Trainers/Branch Manager
- custom groups (Super Admin, Administrator, Finance, Backoffice, …) all run
  on the Administrator interface, restricted by their permissions — reflected
  in the groups table, notes, and Add-user dropdown
- ER model: system_group_key enum gains branch_manager; user_group.system_key
  and the access-control note updated
- PRODUCT_SPEC.md: RBAC section rewritten (4 system groups + Admin-interface
  custom groups)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01C1rM739bFjpxKpAnsLyCHD
</commit_message>
<xml_diff>
--- a/SJA_ER_Model.xlsx
+++ b/SJA_ER_Model.xlsx
@@ -688,7 +688,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Menu access and CRUD rights are per user_group (group_menu_permission, group_resource_permission). A user belongs to one group; Students/Parents/Trainers are locked system groups tied to the dedicated interfaces.</t>
+          <t>Menu access and CRUD rights are per user_group (group_menu_permission, group_resource_permission). A user belongs to one group. Students/Parents/Trainers/Branch Manager are locked system groups, each with its own dedicated interface; every other (custom) group uses the Administrator interface restricted by its permissions.</t>
         </is>
       </c>
     </row>
@@ -2328,7 +2328,7 @@
       </c>
       <c r="G22" s="4" t="inlineStr">
         <is>
-          <t>ENUM: student/parent/trainer — set only for the 3 system groups; drives the dedicated interface</t>
+          <t>ENUM: student/parent/trainer/branch_manager — set only for the 4 locked system groups; drives the dedicated interface. NULL for custom groups (they use the Administrator interface)</t>
         </is>
       </c>
     </row>
@@ -11436,12 +11436,12 @@
       </c>
       <c r="B2" s="8" t="inlineStr">
         <is>
-          <t>student, parent, trainer</t>
+          <t>student, parent, trainer, branch_manager</t>
         </is>
       </c>
       <c r="C2" s="32" t="inlineStr">
         <is>
-          <t>user_group.system_key (locked system groups)</t>
+          <t>user_group.system_key (locked system groups, each with its own interface)</t>
         </is>
       </c>
     </row>

</xml_diff>